<commit_message>
update outputs task 8
</commit_message>
<xml_diff>
--- a/nlp_cia/task 6/test_improved_with_predictions.xlsx
+++ b/nlp_cia/task 6/test_improved_with_predictions.xlsx
@@ -22258,11 +22258,11 @@
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>sadness</t>
         </is>
       </c>
       <c r="K397" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="398">

</xml_diff>